<commit_message>
Fasa 1: log masuk nama+PIN (roster hashed), tab Guru untuk guru sahaja, Cuba lagi kekalkan soalan, Cabaran Harian 10 (6/3/1), reset berpusat (progressVersion), lajur aras
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017jXQRTrJZMGLwUYt6fh7W8
</commit_message>
<xml_diff>
--- a/templates/bank_soalan_template.xlsx
+++ b/templates/bank_soalan_template.xlsx
@@ -660,7 +660,7 @@
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ms: muka surat buku teks.    kbat: Y jika soalan aras tinggi/situasi.    aktif: N untuk menyembunyikan soalan tanpa memadamnya.</t>
+          <t>ms: muka surat buku teks.    kbat: Y jika soalan aras tinggi/situasi.    aras: mudah / sederhana / kbat — menentukan campuran Cabaran Harian (6 mudah, 3 sederhana, 1 KBAT).    aktif: N untuk menyembunyikan soalan tanpa memadamnya.</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W228"/>
+  <dimension ref="A1:X228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -765,7 +765,8 @@
     <col width="56" customWidth="1" min="20" max="20"/>
     <col width="6" customWidth="1" min="21" max="21"/>
     <col width="6" customWidth="1" min="22" max="22"/>
-    <col width="6" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="6" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -880,6 +881,11 @@
         </is>
       </c>
       <c r="W1" s="5" t="inlineStr">
+        <is>
+          <t>aras</t>
+        </is>
+      </c>
+      <c r="X1" s="5" t="inlineStr">
         <is>
           <t>aktif</t>
         </is>
@@ -962,6 +968,11 @@
       </c>
       <c r="W2" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X2" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1039,6 +1050,11 @@
       </c>
       <c r="W3" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X3" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1120,6 +1136,11 @@
       </c>
       <c r="W4" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1201,6 +1222,11 @@
       </c>
       <c r="W5" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X5" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1282,6 +1308,11 @@
       </c>
       <c r="W6" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X6" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1351,6 +1382,11 @@
       </c>
       <c r="W7" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X7" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1427,6 +1463,11 @@
         </is>
       </c>
       <c r="W8" s="6" t="inlineStr">
+        <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X8" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1509,6 +1550,11 @@
       </c>
       <c r="W9" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X9" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1586,6 +1632,11 @@
       </c>
       <c r="W10" s="6" t="inlineStr">
         <is>
+          <t>kbat</t>
+        </is>
+      </c>
+      <c r="X10" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1655,6 +1706,11 @@
       </c>
       <c r="W11" s="6" t="inlineStr">
         <is>
+          <t>kbat</t>
+        </is>
+      </c>
+      <c r="X11" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1736,6 +1792,11 @@
       </c>
       <c r="W12" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X12" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1817,6 +1878,11 @@
       </c>
       <c r="W13" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X13" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1878,6 +1944,11 @@
       </c>
       <c r="W14" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X14" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1939,6 +2010,11 @@
       </c>
       <c r="W15" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X15" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2000,6 +2076,11 @@
       </c>
       <c r="W16" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X16" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2061,6 +2142,11 @@
       </c>
       <c r="W17" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X17" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2122,6 +2208,11 @@
       </c>
       <c r="W18" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X18" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2183,6 +2274,11 @@
       </c>
       <c r="W19" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X19" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2259,6 +2355,11 @@
         </is>
       </c>
       <c r="W20" s="6" t="inlineStr">
+        <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X20" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2333,6 +2434,11 @@
       </c>
       <c r="W21" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X21" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2410,6 +2516,11 @@
       </c>
       <c r="W22" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X22" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2487,6 +2598,11 @@
       </c>
       <c r="W23" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X23" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2564,6 +2680,11 @@
       </c>
       <c r="W24" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X24" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2641,6 +2762,11 @@
       </c>
       <c r="W25" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X25" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2718,6 +2844,11 @@
       </c>
       <c r="W26" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X26" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2795,6 +2926,11 @@
       </c>
       <c r="W27" s="6" t="inlineStr">
         <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="X27" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2871,6 +3007,11 @@
         </is>
       </c>
       <c r="W28" s="6" t="inlineStr">
+        <is>
+          <t>kbat</t>
+        </is>
+      </c>
+      <c r="X28" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2900,6 +3041,7 @@
       <c r="U29" s="8" t="n"/>
       <c r="V29" s="8" t="n"/>
       <c r="W29" s="8" t="n"/>
+      <c r="X29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n"/>
@@ -2925,6 +3067,7 @@
       <c r="U30" s="8" t="n"/>
       <c r="V30" s="8" t="n"/>
       <c r="W30" s="8" t="n"/>
+      <c r="X30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n"/>
@@ -2950,6 +3093,7 @@
       <c r="U31" s="8" t="n"/>
       <c r="V31" s="8" t="n"/>
       <c r="W31" s="8" t="n"/>
+      <c r="X31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n"/>
@@ -2975,6 +3119,7 @@
       <c r="U32" s="8" t="n"/>
       <c r="V32" s="8" t="n"/>
       <c r="W32" s="8" t="n"/>
+      <c r="X32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n"/>
@@ -3000,6 +3145,7 @@
       <c r="U33" s="8" t="n"/>
       <c r="V33" s="8" t="n"/>
       <c r="W33" s="8" t="n"/>
+      <c r="X33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n"/>
@@ -3025,6 +3171,7 @@
       <c r="U34" s="8" t="n"/>
       <c r="V34" s="8" t="n"/>
       <c r="W34" s="8" t="n"/>
+      <c r="X34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n"/>
@@ -3050,6 +3197,7 @@
       <c r="U35" s="8" t="n"/>
       <c r="V35" s="8" t="n"/>
       <c r="W35" s="8" t="n"/>
+      <c r="X35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n"/>
@@ -3075,6 +3223,7 @@
       <c r="U36" s="8" t="n"/>
       <c r="V36" s="8" t="n"/>
       <c r="W36" s="8" t="n"/>
+      <c r="X36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n"/>
@@ -3100,6 +3249,7 @@
       <c r="U37" s="8" t="n"/>
       <c r="V37" s="8" t="n"/>
       <c r="W37" s="8" t="n"/>
+      <c r="X37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n"/>
@@ -3125,6 +3275,7 @@
       <c r="U38" s="8" t="n"/>
       <c r="V38" s="8" t="n"/>
       <c r="W38" s="8" t="n"/>
+      <c r="X38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n"/>
@@ -3150,6 +3301,7 @@
       <c r="U39" s="8" t="n"/>
       <c r="V39" s="8" t="n"/>
       <c r="W39" s="8" t="n"/>
+      <c r="X39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n"/>
@@ -3175,6 +3327,7 @@
       <c r="U40" s="8" t="n"/>
       <c r="V40" s="8" t="n"/>
       <c r="W40" s="8" t="n"/>
+      <c r="X40" s="8" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n"/>
@@ -3200,6 +3353,7 @@
       <c r="U41" s="8" t="n"/>
       <c r="V41" s="8" t="n"/>
       <c r="W41" s="8" t="n"/>
+      <c r="X41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n"/>
@@ -3225,6 +3379,7 @@
       <c r="U42" s="8" t="n"/>
       <c r="V42" s="8" t="n"/>
       <c r="W42" s="8" t="n"/>
+      <c r="X42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n"/>
@@ -3250,6 +3405,7 @@
       <c r="U43" s="8" t="n"/>
       <c r="V43" s="8" t="n"/>
       <c r="W43" s="8" t="n"/>
+      <c r="X43" s="8" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n"/>
@@ -3275,6 +3431,7 @@
       <c r="U44" s="8" t="n"/>
       <c r="V44" s="8" t="n"/>
       <c r="W44" s="8" t="n"/>
+      <c r="X44" s="8" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="n"/>
@@ -3300,6 +3457,7 @@
       <c r="U45" s="8" t="n"/>
       <c r="V45" s="8" t="n"/>
       <c r="W45" s="8" t="n"/>
+      <c r="X45" s="8" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n"/>
@@ -3325,6 +3483,7 @@
       <c r="U46" s="8" t="n"/>
       <c r="V46" s="8" t="n"/>
       <c r="W46" s="8" t="n"/>
+      <c r="X46" s="8" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n"/>
@@ -3350,6 +3509,7 @@
       <c r="U47" s="8" t="n"/>
       <c r="V47" s="8" t="n"/>
       <c r="W47" s="8" t="n"/>
+      <c r="X47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n"/>
@@ -3375,6 +3535,7 @@
       <c r="U48" s="8" t="n"/>
       <c r="V48" s="8" t="n"/>
       <c r="W48" s="8" t="n"/>
+      <c r="X48" s="8" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
@@ -3400,6 +3561,7 @@
       <c r="U49" s="8" t="n"/>
       <c r="V49" s="8" t="n"/>
       <c r="W49" s="8" t="n"/>
+      <c r="X49" s="8" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n"/>
@@ -3425,6 +3587,7 @@
       <c r="U50" s="8" t="n"/>
       <c r="V50" s="8" t="n"/>
       <c r="W50" s="8" t="n"/>
+      <c r="X50" s="8" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n"/>
@@ -3450,6 +3613,7 @@
       <c r="U51" s="8" t="n"/>
       <c r="V51" s="8" t="n"/>
       <c r="W51" s="8" t="n"/>
+      <c r="X51" s="8" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n"/>
@@ -3475,6 +3639,7 @@
       <c r="U52" s="8" t="n"/>
       <c r="V52" s="8" t="n"/>
       <c r="W52" s="8" t="n"/>
+      <c r="X52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n"/>
@@ -3500,6 +3665,7 @@
       <c r="U53" s="8" t="n"/>
       <c r="V53" s="8" t="n"/>
       <c r="W53" s="8" t="n"/>
+      <c r="X53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n"/>
@@ -3525,6 +3691,7 @@
       <c r="U54" s="8" t="n"/>
       <c r="V54" s="8" t="n"/>
       <c r="W54" s="8" t="n"/>
+      <c r="X54" s="8" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n"/>
@@ -3550,6 +3717,7 @@
       <c r="U55" s="8" t="n"/>
       <c r="V55" s="8" t="n"/>
       <c r="W55" s="8" t="n"/>
+      <c r="X55" s="8" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="n"/>
@@ -3575,6 +3743,7 @@
       <c r="U56" s="8" t="n"/>
       <c r="V56" s="8" t="n"/>
       <c r="W56" s="8" t="n"/>
+      <c r="X56" s="8" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n"/>
@@ -3600,6 +3769,7 @@
       <c r="U57" s="8" t="n"/>
       <c r="V57" s="8" t="n"/>
       <c r="W57" s="8" t="n"/>
+      <c r="X57" s="8" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n"/>
@@ -3625,6 +3795,7 @@
       <c r="U58" s="8" t="n"/>
       <c r="V58" s="8" t="n"/>
       <c r="W58" s="8" t="n"/>
+      <c r="X58" s="8" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n"/>
@@ -3650,6 +3821,7 @@
       <c r="U59" s="8" t="n"/>
       <c r="V59" s="8" t="n"/>
       <c r="W59" s="8" t="n"/>
+      <c r="X59" s="8" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n"/>
@@ -3675,6 +3847,7 @@
       <c r="U60" s="8" t="n"/>
       <c r="V60" s="8" t="n"/>
       <c r="W60" s="8" t="n"/>
+      <c r="X60" s="8" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n"/>
@@ -3700,6 +3873,7 @@
       <c r="U61" s="8" t="n"/>
       <c r="V61" s="8" t="n"/>
       <c r="W61" s="8" t="n"/>
+      <c r="X61" s="8" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n"/>
@@ -3725,6 +3899,7 @@
       <c r="U62" s="8" t="n"/>
       <c r="V62" s="8" t="n"/>
       <c r="W62" s="8" t="n"/>
+      <c r="X62" s="8" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n"/>
@@ -3750,6 +3925,7 @@
       <c r="U63" s="8" t="n"/>
       <c r="V63" s="8" t="n"/>
       <c r="W63" s="8" t="n"/>
+      <c r="X63" s="8" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="8" t="n"/>
@@ -3775,6 +3951,7 @@
       <c r="U64" s="8" t="n"/>
       <c r="V64" s="8" t="n"/>
       <c r="W64" s="8" t="n"/>
+      <c r="X64" s="8" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n"/>
@@ -3800,6 +3977,7 @@
       <c r="U65" s="8" t="n"/>
       <c r="V65" s="8" t="n"/>
       <c r="W65" s="8" t="n"/>
+      <c r="X65" s="8" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n"/>
@@ -3825,6 +4003,7 @@
       <c r="U66" s="8" t="n"/>
       <c r="V66" s="8" t="n"/>
       <c r="W66" s="8" t="n"/>
+      <c r="X66" s="8" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n"/>
@@ -3850,6 +4029,7 @@
       <c r="U67" s="8" t="n"/>
       <c r="V67" s="8" t="n"/>
       <c r="W67" s="8" t="n"/>
+      <c r="X67" s="8" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n"/>
@@ -3875,6 +4055,7 @@
       <c r="U68" s="8" t="n"/>
       <c r="V68" s="8" t="n"/>
       <c r="W68" s="8" t="n"/>
+      <c r="X68" s="8" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n"/>
@@ -3900,6 +4081,7 @@
       <c r="U69" s="8" t="n"/>
       <c r="V69" s="8" t="n"/>
       <c r="W69" s="8" t="n"/>
+      <c r="X69" s="8" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n"/>
@@ -3925,6 +4107,7 @@
       <c r="U70" s="8" t="n"/>
       <c r="V70" s="8" t="n"/>
       <c r="W70" s="8" t="n"/>
+      <c r="X70" s="8" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n"/>
@@ -3950,6 +4133,7 @@
       <c r="U71" s="8" t="n"/>
       <c r="V71" s="8" t="n"/>
       <c r="W71" s="8" t="n"/>
+      <c r="X71" s="8" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n"/>
@@ -3975,6 +4159,7 @@
       <c r="U72" s="8" t="n"/>
       <c r="V72" s="8" t="n"/>
       <c r="W72" s="8" t="n"/>
+      <c r="X72" s="8" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="8" t="n"/>
@@ -4000,6 +4185,7 @@
       <c r="U73" s="8" t="n"/>
       <c r="V73" s="8" t="n"/>
       <c r="W73" s="8" t="n"/>
+      <c r="X73" s="8" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="8" t="n"/>
@@ -4025,6 +4211,7 @@
       <c r="U74" s="8" t="n"/>
       <c r="V74" s="8" t="n"/>
       <c r="W74" s="8" t="n"/>
+      <c r="X74" s="8" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n"/>
@@ -4050,6 +4237,7 @@
       <c r="U75" s="8" t="n"/>
       <c r="V75" s="8" t="n"/>
       <c r="W75" s="8" t="n"/>
+      <c r="X75" s="8" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n"/>
@@ -4075,6 +4263,7 @@
       <c r="U76" s="8" t="n"/>
       <c r="V76" s="8" t="n"/>
       <c r="W76" s="8" t="n"/>
+      <c r="X76" s="8" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n"/>
@@ -4100,6 +4289,7 @@
       <c r="U77" s="8" t="n"/>
       <c r="V77" s="8" t="n"/>
       <c r="W77" s="8" t="n"/>
+      <c r="X77" s="8" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n"/>
@@ -4125,6 +4315,7 @@
       <c r="U78" s="8" t="n"/>
       <c r="V78" s="8" t="n"/>
       <c r="W78" s="8" t="n"/>
+      <c r="X78" s="8" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n"/>
@@ -4150,6 +4341,7 @@
       <c r="U79" s="8" t="n"/>
       <c r="V79" s="8" t="n"/>
       <c r="W79" s="8" t="n"/>
+      <c r="X79" s="8" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n"/>
@@ -4175,6 +4367,7 @@
       <c r="U80" s="8" t="n"/>
       <c r="V80" s="8" t="n"/>
       <c r="W80" s="8" t="n"/>
+      <c r="X80" s="8" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="8" t="n"/>
@@ -4200,6 +4393,7 @@
       <c r="U81" s="8" t="n"/>
       <c r="V81" s="8" t="n"/>
       <c r="W81" s="8" t="n"/>
+      <c r="X81" s="8" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n"/>
@@ -4225,6 +4419,7 @@
       <c r="U82" s="8" t="n"/>
       <c r="V82" s="8" t="n"/>
       <c r="W82" s="8" t="n"/>
+      <c r="X82" s="8" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="8" t="n"/>
@@ -4250,6 +4445,7 @@
       <c r="U83" s="8" t="n"/>
       <c r="V83" s="8" t="n"/>
       <c r="W83" s="8" t="n"/>
+      <c r="X83" s="8" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="8" t="n"/>
@@ -4275,6 +4471,7 @@
       <c r="U84" s="8" t="n"/>
       <c r="V84" s="8" t="n"/>
       <c r="W84" s="8" t="n"/>
+      <c r="X84" s="8" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n"/>
@@ -4300,6 +4497,7 @@
       <c r="U85" s="8" t="n"/>
       <c r="V85" s="8" t="n"/>
       <c r="W85" s="8" t="n"/>
+      <c r="X85" s="8" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="8" t="n"/>
@@ -4325,6 +4523,7 @@
       <c r="U86" s="8" t="n"/>
       <c r="V86" s="8" t="n"/>
       <c r="W86" s="8" t="n"/>
+      <c r="X86" s="8" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="8" t="n"/>
@@ -4350,6 +4549,7 @@
       <c r="U87" s="8" t="n"/>
       <c r="V87" s="8" t="n"/>
       <c r="W87" s="8" t="n"/>
+      <c r="X87" s="8" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="8" t="n"/>
@@ -4375,6 +4575,7 @@
       <c r="U88" s="8" t="n"/>
       <c r="V88" s="8" t="n"/>
       <c r="W88" s="8" t="n"/>
+      <c r="X88" s="8" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="8" t="n"/>
@@ -4400,6 +4601,7 @@
       <c r="U89" s="8" t="n"/>
       <c r="V89" s="8" t="n"/>
       <c r="W89" s="8" t="n"/>
+      <c r="X89" s="8" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="8" t="n"/>
@@ -4425,6 +4627,7 @@
       <c r="U90" s="8" t="n"/>
       <c r="V90" s="8" t="n"/>
       <c r="W90" s="8" t="n"/>
+      <c r="X90" s="8" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="8" t="n"/>
@@ -4450,6 +4653,7 @@
       <c r="U91" s="8" t="n"/>
       <c r="V91" s="8" t="n"/>
       <c r="W91" s="8" t="n"/>
+      <c r="X91" s="8" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="8" t="n"/>
@@ -4475,6 +4679,7 @@
       <c r="U92" s="8" t="n"/>
       <c r="V92" s="8" t="n"/>
       <c r="W92" s="8" t="n"/>
+      <c r="X92" s="8" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="8" t="n"/>
@@ -4500,6 +4705,7 @@
       <c r="U93" s="8" t="n"/>
       <c r="V93" s="8" t="n"/>
       <c r="W93" s="8" t="n"/>
+      <c r="X93" s="8" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="8" t="n"/>
@@ -4525,6 +4731,7 @@
       <c r="U94" s="8" t="n"/>
       <c r="V94" s="8" t="n"/>
       <c r="W94" s="8" t="n"/>
+      <c r="X94" s="8" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="8" t="n"/>
@@ -4550,6 +4757,7 @@
       <c r="U95" s="8" t="n"/>
       <c r="V95" s="8" t="n"/>
       <c r="W95" s="8" t="n"/>
+      <c r="X95" s="8" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="8" t="n"/>
@@ -4575,6 +4783,7 @@
       <c r="U96" s="8" t="n"/>
       <c r="V96" s="8" t="n"/>
       <c r="W96" s="8" t="n"/>
+      <c r="X96" s="8" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="8" t="n"/>
@@ -4600,6 +4809,7 @@
       <c r="U97" s="8" t="n"/>
       <c r="V97" s="8" t="n"/>
       <c r="W97" s="8" t="n"/>
+      <c r="X97" s="8" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="8" t="n"/>
@@ -4625,6 +4835,7 @@
       <c r="U98" s="8" t="n"/>
       <c r="V98" s="8" t="n"/>
       <c r="W98" s="8" t="n"/>
+      <c r="X98" s="8" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="8" t="n"/>
@@ -4650,6 +4861,7 @@
       <c r="U99" s="8" t="n"/>
       <c r="V99" s="8" t="n"/>
       <c r="W99" s="8" t="n"/>
+      <c r="X99" s="8" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="8" t="n"/>
@@ -4675,6 +4887,7 @@
       <c r="U100" s="8" t="n"/>
       <c r="V100" s="8" t="n"/>
       <c r="W100" s="8" t="n"/>
+      <c r="X100" s="8" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="8" t="n"/>
@@ -4700,6 +4913,7 @@
       <c r="U101" s="8" t="n"/>
       <c r="V101" s="8" t="n"/>
       <c r="W101" s="8" t="n"/>
+      <c r="X101" s="8" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="8" t="n"/>
@@ -4725,6 +4939,7 @@
       <c r="U102" s="8" t="n"/>
       <c r="V102" s="8" t="n"/>
       <c r="W102" s="8" t="n"/>
+      <c r="X102" s="8" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="8" t="n"/>
@@ -4750,6 +4965,7 @@
       <c r="U103" s="8" t="n"/>
       <c r="V103" s="8" t="n"/>
       <c r="W103" s="8" t="n"/>
+      <c r="X103" s="8" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="8" t="n"/>
@@ -4775,6 +4991,7 @@
       <c r="U104" s="8" t="n"/>
       <c r="V104" s="8" t="n"/>
       <c r="W104" s="8" t="n"/>
+      <c r="X104" s="8" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="8" t="n"/>
@@ -4800,6 +5017,7 @@
       <c r="U105" s="8" t="n"/>
       <c r="V105" s="8" t="n"/>
       <c r="W105" s="8" t="n"/>
+      <c r="X105" s="8" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="8" t="n"/>
@@ -4825,6 +5043,7 @@
       <c r="U106" s="8" t="n"/>
       <c r="V106" s="8" t="n"/>
       <c r="W106" s="8" t="n"/>
+      <c r="X106" s="8" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="8" t="n"/>
@@ -4850,6 +5069,7 @@
       <c r="U107" s="8" t="n"/>
       <c r="V107" s="8" t="n"/>
       <c r="W107" s="8" t="n"/>
+      <c r="X107" s="8" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="8" t="n"/>
@@ -4875,6 +5095,7 @@
       <c r="U108" s="8" t="n"/>
       <c r="V108" s="8" t="n"/>
       <c r="W108" s="8" t="n"/>
+      <c r="X108" s="8" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="8" t="n"/>
@@ -4900,6 +5121,7 @@
       <c r="U109" s="8" t="n"/>
       <c r="V109" s="8" t="n"/>
       <c r="W109" s="8" t="n"/>
+      <c r="X109" s="8" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="8" t="n"/>
@@ -4925,6 +5147,7 @@
       <c r="U110" s="8" t="n"/>
       <c r="V110" s="8" t="n"/>
       <c r="W110" s="8" t="n"/>
+      <c r="X110" s="8" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="8" t="n"/>
@@ -4950,6 +5173,7 @@
       <c r="U111" s="8" t="n"/>
       <c r="V111" s="8" t="n"/>
       <c r="W111" s="8" t="n"/>
+      <c r="X111" s="8" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="8" t="n"/>
@@ -4975,6 +5199,7 @@
       <c r="U112" s="8" t="n"/>
       <c r="V112" s="8" t="n"/>
       <c r="W112" s="8" t="n"/>
+      <c r="X112" s="8" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="8" t="n"/>
@@ -5000,6 +5225,7 @@
       <c r="U113" s="8" t="n"/>
       <c r="V113" s="8" t="n"/>
       <c r="W113" s="8" t="n"/>
+      <c r="X113" s="8" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="8" t="n"/>
@@ -5025,6 +5251,7 @@
       <c r="U114" s="8" t="n"/>
       <c r="V114" s="8" t="n"/>
       <c r="W114" s="8" t="n"/>
+      <c r="X114" s="8" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="8" t="n"/>
@@ -5050,6 +5277,7 @@
       <c r="U115" s="8" t="n"/>
       <c r="V115" s="8" t="n"/>
       <c r="W115" s="8" t="n"/>
+      <c r="X115" s="8" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="8" t="n"/>
@@ -5075,6 +5303,7 @@
       <c r="U116" s="8" t="n"/>
       <c r="V116" s="8" t="n"/>
       <c r="W116" s="8" t="n"/>
+      <c r="X116" s="8" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="8" t="n"/>
@@ -5100,6 +5329,7 @@
       <c r="U117" s="8" t="n"/>
       <c r="V117" s="8" t="n"/>
       <c r="W117" s="8" t="n"/>
+      <c r="X117" s="8" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="8" t="n"/>
@@ -5125,6 +5355,7 @@
       <c r="U118" s="8" t="n"/>
       <c r="V118" s="8" t="n"/>
       <c r="W118" s="8" t="n"/>
+      <c r="X118" s="8" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="8" t="n"/>
@@ -5150,6 +5381,7 @@
       <c r="U119" s="8" t="n"/>
       <c r="V119" s="8" t="n"/>
       <c r="W119" s="8" t="n"/>
+      <c r="X119" s="8" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="8" t="n"/>
@@ -5175,6 +5407,7 @@
       <c r="U120" s="8" t="n"/>
       <c r="V120" s="8" t="n"/>
       <c r="W120" s="8" t="n"/>
+      <c r="X120" s="8" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="8" t="n"/>
@@ -5200,6 +5433,7 @@
       <c r="U121" s="8" t="n"/>
       <c r="V121" s="8" t="n"/>
       <c r="W121" s="8" t="n"/>
+      <c r="X121" s="8" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="8" t="n"/>
@@ -5225,6 +5459,7 @@
       <c r="U122" s="8" t="n"/>
       <c r="V122" s="8" t="n"/>
       <c r="W122" s="8" t="n"/>
+      <c r="X122" s="8" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="8" t="n"/>
@@ -5250,6 +5485,7 @@
       <c r="U123" s="8" t="n"/>
       <c r="V123" s="8" t="n"/>
       <c r="W123" s="8" t="n"/>
+      <c r="X123" s="8" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="8" t="n"/>
@@ -5275,6 +5511,7 @@
       <c r="U124" s="8" t="n"/>
       <c r="V124" s="8" t="n"/>
       <c r="W124" s="8" t="n"/>
+      <c r="X124" s="8" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="8" t="n"/>
@@ -5300,6 +5537,7 @@
       <c r="U125" s="8" t="n"/>
       <c r="V125" s="8" t="n"/>
       <c r="W125" s="8" t="n"/>
+      <c r="X125" s="8" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="8" t="n"/>
@@ -5325,6 +5563,7 @@
       <c r="U126" s="8" t="n"/>
       <c r="V126" s="8" t="n"/>
       <c r="W126" s="8" t="n"/>
+      <c r="X126" s="8" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="8" t="n"/>
@@ -5350,6 +5589,7 @@
       <c r="U127" s="8" t="n"/>
       <c r="V127" s="8" t="n"/>
       <c r="W127" s="8" t="n"/>
+      <c r="X127" s="8" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="8" t="n"/>
@@ -5375,6 +5615,7 @@
       <c r="U128" s="8" t="n"/>
       <c r="V128" s="8" t="n"/>
       <c r="W128" s="8" t="n"/>
+      <c r="X128" s="8" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="8" t="n"/>
@@ -5400,6 +5641,7 @@
       <c r="U129" s="8" t="n"/>
       <c r="V129" s="8" t="n"/>
       <c r="W129" s="8" t="n"/>
+      <c r="X129" s="8" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="8" t="n"/>
@@ -5425,6 +5667,7 @@
       <c r="U130" s="8" t="n"/>
       <c r="V130" s="8" t="n"/>
       <c r="W130" s="8" t="n"/>
+      <c r="X130" s="8" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="8" t="n"/>
@@ -5450,6 +5693,7 @@
       <c r="U131" s="8" t="n"/>
       <c r="V131" s="8" t="n"/>
       <c r="W131" s="8" t="n"/>
+      <c r="X131" s="8" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="8" t="n"/>
@@ -5475,6 +5719,7 @@
       <c r="U132" s="8" t="n"/>
       <c r="V132" s="8" t="n"/>
       <c r="W132" s="8" t="n"/>
+      <c r="X132" s="8" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="8" t="n"/>
@@ -5500,6 +5745,7 @@
       <c r="U133" s="8" t="n"/>
       <c r="V133" s="8" t="n"/>
       <c r="W133" s="8" t="n"/>
+      <c r="X133" s="8" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="8" t="n"/>
@@ -5525,6 +5771,7 @@
       <c r="U134" s="8" t="n"/>
       <c r="V134" s="8" t="n"/>
       <c r="W134" s="8" t="n"/>
+      <c r="X134" s="8" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="8" t="n"/>
@@ -5550,6 +5797,7 @@
       <c r="U135" s="8" t="n"/>
       <c r="V135" s="8" t="n"/>
       <c r="W135" s="8" t="n"/>
+      <c r="X135" s="8" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="8" t="n"/>
@@ -5575,6 +5823,7 @@
       <c r="U136" s="8" t="n"/>
       <c r="V136" s="8" t="n"/>
       <c r="W136" s="8" t="n"/>
+      <c r="X136" s="8" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="8" t="n"/>
@@ -5600,6 +5849,7 @@
       <c r="U137" s="8" t="n"/>
       <c r="V137" s="8" t="n"/>
       <c r="W137" s="8" t="n"/>
+      <c r="X137" s="8" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="8" t="n"/>
@@ -5625,6 +5875,7 @@
       <c r="U138" s="8" t="n"/>
       <c r="V138" s="8" t="n"/>
       <c r="W138" s="8" t="n"/>
+      <c r="X138" s="8" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="8" t="n"/>
@@ -5650,6 +5901,7 @@
       <c r="U139" s="8" t="n"/>
       <c r="V139" s="8" t="n"/>
       <c r="W139" s="8" t="n"/>
+      <c r="X139" s="8" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="8" t="n"/>
@@ -5675,6 +5927,7 @@
       <c r="U140" s="8" t="n"/>
       <c r="V140" s="8" t="n"/>
       <c r="W140" s="8" t="n"/>
+      <c r="X140" s="8" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="8" t="n"/>
@@ -5700,6 +5953,7 @@
       <c r="U141" s="8" t="n"/>
       <c r="V141" s="8" t="n"/>
       <c r="W141" s="8" t="n"/>
+      <c r="X141" s="8" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="8" t="n"/>
@@ -5725,6 +5979,7 @@
       <c r="U142" s="8" t="n"/>
       <c r="V142" s="8" t="n"/>
       <c r="W142" s="8" t="n"/>
+      <c r="X142" s="8" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="8" t="n"/>
@@ -5750,6 +6005,7 @@
       <c r="U143" s="8" t="n"/>
       <c r="V143" s="8" t="n"/>
       <c r="W143" s="8" t="n"/>
+      <c r="X143" s="8" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="8" t="n"/>
@@ -5775,6 +6031,7 @@
       <c r="U144" s="8" t="n"/>
       <c r="V144" s="8" t="n"/>
       <c r="W144" s="8" t="n"/>
+      <c r="X144" s="8" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="8" t="n"/>
@@ -5800,6 +6057,7 @@
       <c r="U145" s="8" t="n"/>
       <c r="V145" s="8" t="n"/>
       <c r="W145" s="8" t="n"/>
+      <c r="X145" s="8" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="8" t="n"/>
@@ -5825,6 +6083,7 @@
       <c r="U146" s="8" t="n"/>
       <c r="V146" s="8" t="n"/>
       <c r="W146" s="8" t="n"/>
+      <c r="X146" s="8" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="8" t="n"/>
@@ -5850,6 +6109,7 @@
       <c r="U147" s="8" t="n"/>
       <c r="V147" s="8" t="n"/>
       <c r="W147" s="8" t="n"/>
+      <c r="X147" s="8" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="8" t="n"/>
@@ -5875,6 +6135,7 @@
       <c r="U148" s="8" t="n"/>
       <c r="V148" s="8" t="n"/>
       <c r="W148" s="8" t="n"/>
+      <c r="X148" s="8" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="8" t="n"/>
@@ -5900,6 +6161,7 @@
       <c r="U149" s="8" t="n"/>
       <c r="V149" s="8" t="n"/>
       <c r="W149" s="8" t="n"/>
+      <c r="X149" s="8" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="8" t="n"/>
@@ -5925,6 +6187,7 @@
       <c r="U150" s="8" t="n"/>
       <c r="V150" s="8" t="n"/>
       <c r="W150" s="8" t="n"/>
+      <c r="X150" s="8" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="8" t="n"/>
@@ -5950,6 +6213,7 @@
       <c r="U151" s="8" t="n"/>
       <c r="V151" s="8" t="n"/>
       <c r="W151" s="8" t="n"/>
+      <c r="X151" s="8" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="8" t="n"/>
@@ -5975,6 +6239,7 @@
       <c r="U152" s="8" t="n"/>
       <c r="V152" s="8" t="n"/>
       <c r="W152" s="8" t="n"/>
+      <c r="X152" s="8" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="8" t="n"/>
@@ -6000,6 +6265,7 @@
       <c r="U153" s="8" t="n"/>
       <c r="V153" s="8" t="n"/>
       <c r="W153" s="8" t="n"/>
+      <c r="X153" s="8" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="8" t="n"/>
@@ -6025,6 +6291,7 @@
       <c r="U154" s="8" t="n"/>
       <c r="V154" s="8" t="n"/>
       <c r="W154" s="8" t="n"/>
+      <c r="X154" s="8" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="8" t="n"/>
@@ -6050,6 +6317,7 @@
       <c r="U155" s="8" t="n"/>
       <c r="V155" s="8" t="n"/>
       <c r="W155" s="8" t="n"/>
+      <c r="X155" s="8" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="8" t="n"/>
@@ -6075,6 +6343,7 @@
       <c r="U156" s="8" t="n"/>
       <c r="V156" s="8" t="n"/>
       <c r="W156" s="8" t="n"/>
+      <c r="X156" s="8" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="8" t="n"/>
@@ -6100,6 +6369,7 @@
       <c r="U157" s="8" t="n"/>
       <c r="V157" s="8" t="n"/>
       <c r="W157" s="8" t="n"/>
+      <c r="X157" s="8" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="8" t="n"/>
@@ -6125,6 +6395,7 @@
       <c r="U158" s="8" t="n"/>
       <c r="V158" s="8" t="n"/>
       <c r="W158" s="8" t="n"/>
+      <c r="X158" s="8" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="8" t="n"/>
@@ -6150,6 +6421,7 @@
       <c r="U159" s="8" t="n"/>
       <c r="V159" s="8" t="n"/>
       <c r="W159" s="8" t="n"/>
+      <c r="X159" s="8" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="8" t="n"/>
@@ -6175,6 +6447,7 @@
       <c r="U160" s="8" t="n"/>
       <c r="V160" s="8" t="n"/>
       <c r="W160" s="8" t="n"/>
+      <c r="X160" s="8" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="8" t="n"/>
@@ -6200,6 +6473,7 @@
       <c r="U161" s="8" t="n"/>
       <c r="V161" s="8" t="n"/>
       <c r="W161" s="8" t="n"/>
+      <c r="X161" s="8" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="8" t="n"/>
@@ -6225,6 +6499,7 @@
       <c r="U162" s="8" t="n"/>
       <c r="V162" s="8" t="n"/>
       <c r="W162" s="8" t="n"/>
+      <c r="X162" s="8" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="8" t="n"/>
@@ -6250,6 +6525,7 @@
       <c r="U163" s="8" t="n"/>
       <c r="V163" s="8" t="n"/>
       <c r="W163" s="8" t="n"/>
+      <c r="X163" s="8" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="8" t="n"/>
@@ -6275,6 +6551,7 @@
       <c r="U164" s="8" t="n"/>
       <c r="V164" s="8" t="n"/>
       <c r="W164" s="8" t="n"/>
+      <c r="X164" s="8" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="8" t="n"/>
@@ -6300,6 +6577,7 @@
       <c r="U165" s="8" t="n"/>
       <c r="V165" s="8" t="n"/>
       <c r="W165" s="8" t="n"/>
+      <c r="X165" s="8" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="8" t="n"/>
@@ -6325,6 +6603,7 @@
       <c r="U166" s="8" t="n"/>
       <c r="V166" s="8" t="n"/>
       <c r="W166" s="8" t="n"/>
+      <c r="X166" s="8" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="8" t="n"/>
@@ -6350,6 +6629,7 @@
       <c r="U167" s="8" t="n"/>
       <c r="V167" s="8" t="n"/>
       <c r="W167" s="8" t="n"/>
+      <c r="X167" s="8" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="8" t="n"/>
@@ -6375,6 +6655,7 @@
       <c r="U168" s="8" t="n"/>
       <c r="V168" s="8" t="n"/>
       <c r="W168" s="8" t="n"/>
+      <c r="X168" s="8" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="8" t="n"/>
@@ -6400,6 +6681,7 @@
       <c r="U169" s="8" t="n"/>
       <c r="V169" s="8" t="n"/>
       <c r="W169" s="8" t="n"/>
+      <c r="X169" s="8" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="8" t="n"/>
@@ -6425,6 +6707,7 @@
       <c r="U170" s="8" t="n"/>
       <c r="V170" s="8" t="n"/>
       <c r="W170" s="8" t="n"/>
+      <c r="X170" s="8" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="8" t="n"/>
@@ -6450,6 +6733,7 @@
       <c r="U171" s="8" t="n"/>
       <c r="V171" s="8" t="n"/>
       <c r="W171" s="8" t="n"/>
+      <c r="X171" s="8" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="8" t="n"/>
@@ -6475,6 +6759,7 @@
       <c r="U172" s="8" t="n"/>
       <c r="V172" s="8" t="n"/>
       <c r="W172" s="8" t="n"/>
+      <c r="X172" s="8" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="8" t="n"/>
@@ -6500,6 +6785,7 @@
       <c r="U173" s="8" t="n"/>
       <c r="V173" s="8" t="n"/>
       <c r="W173" s="8" t="n"/>
+      <c r="X173" s="8" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="8" t="n"/>
@@ -6525,6 +6811,7 @@
       <c r="U174" s="8" t="n"/>
       <c r="V174" s="8" t="n"/>
       <c r="W174" s="8" t="n"/>
+      <c r="X174" s="8" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="8" t="n"/>
@@ -6550,6 +6837,7 @@
       <c r="U175" s="8" t="n"/>
       <c r="V175" s="8" t="n"/>
       <c r="W175" s="8" t="n"/>
+      <c r="X175" s="8" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="8" t="n"/>
@@ -6575,6 +6863,7 @@
       <c r="U176" s="8" t="n"/>
       <c r="V176" s="8" t="n"/>
       <c r="W176" s="8" t="n"/>
+      <c r="X176" s="8" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="8" t="n"/>
@@ -6600,6 +6889,7 @@
       <c r="U177" s="8" t="n"/>
       <c r="V177" s="8" t="n"/>
       <c r="W177" s="8" t="n"/>
+      <c r="X177" s="8" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="8" t="n"/>
@@ -6625,6 +6915,7 @@
       <c r="U178" s="8" t="n"/>
       <c r="V178" s="8" t="n"/>
       <c r="W178" s="8" t="n"/>
+      <c r="X178" s="8" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="8" t="n"/>
@@ -6650,6 +6941,7 @@
       <c r="U179" s="8" t="n"/>
       <c r="V179" s="8" t="n"/>
       <c r="W179" s="8" t="n"/>
+      <c r="X179" s="8" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="8" t="n"/>
@@ -6675,6 +6967,7 @@
       <c r="U180" s="8" t="n"/>
       <c r="V180" s="8" t="n"/>
       <c r="W180" s="8" t="n"/>
+      <c r="X180" s="8" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="8" t="n"/>
@@ -6700,6 +6993,7 @@
       <c r="U181" s="8" t="n"/>
       <c r="V181" s="8" t="n"/>
       <c r="W181" s="8" t="n"/>
+      <c r="X181" s="8" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="8" t="n"/>
@@ -6725,6 +7019,7 @@
       <c r="U182" s="8" t="n"/>
       <c r="V182" s="8" t="n"/>
       <c r="W182" s="8" t="n"/>
+      <c r="X182" s="8" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="8" t="n"/>
@@ -6750,6 +7045,7 @@
       <c r="U183" s="8" t="n"/>
       <c r="V183" s="8" t="n"/>
       <c r="W183" s="8" t="n"/>
+      <c r="X183" s="8" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="8" t="n"/>
@@ -6775,6 +7071,7 @@
       <c r="U184" s="8" t="n"/>
       <c r="V184" s="8" t="n"/>
       <c r="W184" s="8" t="n"/>
+      <c r="X184" s="8" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="8" t="n"/>
@@ -6800,6 +7097,7 @@
       <c r="U185" s="8" t="n"/>
       <c r="V185" s="8" t="n"/>
       <c r="W185" s="8" t="n"/>
+      <c r="X185" s="8" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="8" t="n"/>
@@ -6825,6 +7123,7 @@
       <c r="U186" s="8" t="n"/>
       <c r="V186" s="8" t="n"/>
       <c r="W186" s="8" t="n"/>
+      <c r="X186" s="8" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="8" t="n"/>
@@ -6850,6 +7149,7 @@
       <c r="U187" s="8" t="n"/>
       <c r="V187" s="8" t="n"/>
       <c r="W187" s="8" t="n"/>
+      <c r="X187" s="8" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="8" t="n"/>
@@ -6875,6 +7175,7 @@
       <c r="U188" s="8" t="n"/>
       <c r="V188" s="8" t="n"/>
       <c r="W188" s="8" t="n"/>
+      <c r="X188" s="8" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="8" t="n"/>
@@ -6900,6 +7201,7 @@
       <c r="U189" s="8" t="n"/>
       <c r="V189" s="8" t="n"/>
       <c r="W189" s="8" t="n"/>
+      <c r="X189" s="8" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="8" t="n"/>
@@ -6925,6 +7227,7 @@
       <c r="U190" s="8" t="n"/>
       <c r="V190" s="8" t="n"/>
       <c r="W190" s="8" t="n"/>
+      <c r="X190" s="8" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="8" t="n"/>
@@ -6950,6 +7253,7 @@
       <c r="U191" s="8" t="n"/>
       <c r="V191" s="8" t="n"/>
       <c r="W191" s="8" t="n"/>
+      <c r="X191" s="8" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="8" t="n"/>
@@ -6975,6 +7279,7 @@
       <c r="U192" s="8" t="n"/>
       <c r="V192" s="8" t="n"/>
       <c r="W192" s="8" t="n"/>
+      <c r="X192" s="8" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="8" t="n"/>
@@ -7000,6 +7305,7 @@
       <c r="U193" s="8" t="n"/>
       <c r="V193" s="8" t="n"/>
       <c r="W193" s="8" t="n"/>
+      <c r="X193" s="8" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="8" t="n"/>
@@ -7025,6 +7331,7 @@
       <c r="U194" s="8" t="n"/>
       <c r="V194" s="8" t="n"/>
       <c r="W194" s="8" t="n"/>
+      <c r="X194" s="8" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="8" t="n"/>
@@ -7050,6 +7357,7 @@
       <c r="U195" s="8" t="n"/>
       <c r="V195" s="8" t="n"/>
       <c r="W195" s="8" t="n"/>
+      <c r="X195" s="8" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="8" t="n"/>
@@ -7075,6 +7383,7 @@
       <c r="U196" s="8" t="n"/>
       <c r="V196" s="8" t="n"/>
       <c r="W196" s="8" t="n"/>
+      <c r="X196" s="8" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="8" t="n"/>
@@ -7100,6 +7409,7 @@
       <c r="U197" s="8" t="n"/>
       <c r="V197" s="8" t="n"/>
       <c r="W197" s="8" t="n"/>
+      <c r="X197" s="8" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="8" t="n"/>
@@ -7125,6 +7435,7 @@
       <c r="U198" s="8" t="n"/>
       <c r="V198" s="8" t="n"/>
       <c r="W198" s="8" t="n"/>
+      <c r="X198" s="8" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="8" t="n"/>
@@ -7150,6 +7461,7 @@
       <c r="U199" s="8" t="n"/>
       <c r="V199" s="8" t="n"/>
       <c r="W199" s="8" t="n"/>
+      <c r="X199" s="8" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="8" t="n"/>
@@ -7175,6 +7487,7 @@
       <c r="U200" s="8" t="n"/>
       <c r="V200" s="8" t="n"/>
       <c r="W200" s="8" t="n"/>
+      <c r="X200" s="8" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="8" t="n"/>
@@ -7200,6 +7513,7 @@
       <c r="U201" s="8" t="n"/>
       <c r="V201" s="8" t="n"/>
       <c r="W201" s="8" t="n"/>
+      <c r="X201" s="8" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="8" t="n"/>
@@ -7225,6 +7539,7 @@
       <c r="U202" s="8" t="n"/>
       <c r="V202" s="8" t="n"/>
       <c r="W202" s="8" t="n"/>
+      <c r="X202" s="8" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="8" t="n"/>
@@ -7250,6 +7565,7 @@
       <c r="U203" s="8" t="n"/>
       <c r="V203" s="8" t="n"/>
       <c r="W203" s="8" t="n"/>
+      <c r="X203" s="8" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="8" t="n"/>
@@ -7275,6 +7591,7 @@
       <c r="U204" s="8" t="n"/>
       <c r="V204" s="8" t="n"/>
       <c r="W204" s="8" t="n"/>
+      <c r="X204" s="8" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="8" t="n"/>
@@ -7300,6 +7617,7 @@
       <c r="U205" s="8" t="n"/>
       <c r="V205" s="8" t="n"/>
       <c r="W205" s="8" t="n"/>
+      <c r="X205" s="8" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="8" t="n"/>
@@ -7325,6 +7643,7 @@
       <c r="U206" s="8" t="n"/>
       <c r="V206" s="8" t="n"/>
       <c r="W206" s="8" t="n"/>
+      <c r="X206" s="8" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="8" t="n"/>
@@ -7350,6 +7669,7 @@
       <c r="U207" s="8" t="n"/>
       <c r="V207" s="8" t="n"/>
       <c r="W207" s="8" t="n"/>
+      <c r="X207" s="8" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="8" t="n"/>
@@ -7375,6 +7695,7 @@
       <c r="U208" s="8" t="n"/>
       <c r="V208" s="8" t="n"/>
       <c r="W208" s="8" t="n"/>
+      <c r="X208" s="8" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="8" t="n"/>
@@ -7400,6 +7721,7 @@
       <c r="U209" s="8" t="n"/>
       <c r="V209" s="8" t="n"/>
       <c r="W209" s="8" t="n"/>
+      <c r="X209" s="8" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="8" t="n"/>
@@ -7425,6 +7747,7 @@
       <c r="U210" s="8" t="n"/>
       <c r="V210" s="8" t="n"/>
       <c r="W210" s="8" t="n"/>
+      <c r="X210" s="8" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="8" t="n"/>
@@ -7450,6 +7773,7 @@
       <c r="U211" s="8" t="n"/>
       <c r="V211" s="8" t="n"/>
       <c r="W211" s="8" t="n"/>
+      <c r="X211" s="8" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="8" t="n"/>
@@ -7475,6 +7799,7 @@
       <c r="U212" s="8" t="n"/>
       <c r="V212" s="8" t="n"/>
       <c r="W212" s="8" t="n"/>
+      <c r="X212" s="8" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="8" t="n"/>
@@ -7500,6 +7825,7 @@
       <c r="U213" s="8" t="n"/>
       <c r="V213" s="8" t="n"/>
       <c r="W213" s="8" t="n"/>
+      <c r="X213" s="8" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="8" t="n"/>
@@ -7525,6 +7851,7 @@
       <c r="U214" s="8" t="n"/>
       <c r="V214" s="8" t="n"/>
       <c r="W214" s="8" t="n"/>
+      <c r="X214" s="8" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="8" t="n"/>
@@ -7550,6 +7877,7 @@
       <c r="U215" s="8" t="n"/>
       <c r="V215" s="8" t="n"/>
       <c r="W215" s="8" t="n"/>
+      <c r="X215" s="8" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="8" t="n"/>
@@ -7575,6 +7903,7 @@
       <c r="U216" s="8" t="n"/>
       <c r="V216" s="8" t="n"/>
       <c r="W216" s="8" t="n"/>
+      <c r="X216" s="8" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="8" t="n"/>
@@ -7600,6 +7929,7 @@
       <c r="U217" s="8" t="n"/>
       <c r="V217" s="8" t="n"/>
       <c r="W217" s="8" t="n"/>
+      <c r="X217" s="8" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="8" t="n"/>
@@ -7625,6 +7955,7 @@
       <c r="U218" s="8" t="n"/>
       <c r="V218" s="8" t="n"/>
       <c r="W218" s="8" t="n"/>
+      <c r="X218" s="8" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="8" t="n"/>
@@ -7650,6 +7981,7 @@
       <c r="U219" s="8" t="n"/>
       <c r="V219" s="8" t="n"/>
       <c r="W219" s="8" t="n"/>
+      <c r="X219" s="8" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="8" t="n"/>
@@ -7675,6 +8007,7 @@
       <c r="U220" s="8" t="n"/>
       <c r="V220" s="8" t="n"/>
       <c r="W220" s="8" t="n"/>
+      <c r="X220" s="8" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="8" t="n"/>
@@ -7700,6 +8033,7 @@
       <c r="U221" s="8" t="n"/>
       <c r="V221" s="8" t="n"/>
       <c r="W221" s="8" t="n"/>
+      <c r="X221" s="8" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="8" t="n"/>
@@ -7725,6 +8059,7 @@
       <c r="U222" s="8" t="n"/>
       <c r="V222" s="8" t="n"/>
       <c r="W222" s="8" t="n"/>
+      <c r="X222" s="8" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="8" t="n"/>
@@ -7750,6 +8085,7 @@
       <c r="U223" s="8" t="n"/>
       <c r="V223" s="8" t="n"/>
       <c r="W223" s="8" t="n"/>
+      <c r="X223" s="8" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="8" t="n"/>
@@ -7775,6 +8111,7 @@
       <c r="U224" s="8" t="n"/>
       <c r="V224" s="8" t="n"/>
       <c r="W224" s="8" t="n"/>
+      <c r="X224" s="8" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="8" t="n"/>
@@ -7800,6 +8137,7 @@
       <c r="U225" s="8" t="n"/>
       <c r="V225" s="8" t="n"/>
       <c r="W225" s="8" t="n"/>
+      <c r="X225" s="8" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="8" t="n"/>
@@ -7825,6 +8163,7 @@
       <c r="U226" s="8" t="n"/>
       <c r="V226" s="8" t="n"/>
       <c r="W226" s="8" t="n"/>
+      <c r="X226" s="8" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="8" t="n"/>
@@ -7850,6 +8189,7 @@
       <c r="U227" s="8" t="n"/>
       <c r="V227" s="8" t="n"/>
       <c r="W227" s="8" t="n"/>
+      <c r="X227" s="8" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="8" t="n"/>
@@ -7875,9 +8215,10 @@
       <c r="U228" s="8" t="n"/>
       <c r="V228" s="8" t="n"/>
       <c r="W228" s="8" t="n"/>
+      <c r="X228" s="8" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation sqref="D2:D228" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"mcq,tf,order,tajwid,fill,jawi"</formula1>
     </dataValidation>
@@ -7888,6 +8229,9 @@
       <formula1>"Y,N"</formula1>
     </dataValidation>
     <dataValidation sqref="W2:W228" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"mudah,sederhana,kbat"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X2:X228" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B228" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">

</xml_diff>